<commit_message>
Isaac Requests, More TBR sims, and TBR sheet updates
</commit_message>
<xml_diff>
--- a/OpenMC_STAR_Model/TBR_sheet.xlsx
+++ b/OpenMC_STAR_Model/TBR_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rocco698/Desktop/Undergrad/Spring_2026/NUCE_431W/NUCE_431W/OpenMC_STAR_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32FD2A7C-9F83-A444-8046-0EBF2291688F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07BBB8C-5FFB-B24C-8FA6-365D2EDBB021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="920" windowWidth="29920" windowHeight="17280" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="32">
   <si>
     <t>Particles</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>PbLi</t>
+  </si>
+  <si>
+    <t>TBR-</t>
+  </si>
+  <si>
+    <t>Above are 17% Li, 83% Pb (at.)</t>
   </si>
 </sst>
 </file>
@@ -324,13 +330,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="3"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="4"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="3" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -339,7 +345,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -678,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21FEB923-94CE-9048-A235-5E054F03F29C}">
-  <dimension ref="A1:AG25"/>
+  <dimension ref="A1:AG27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -691,30 +699,30 @@
       <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="T1" s="7" t="s">
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="T1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="Y1" s="7" t="s">
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="Y1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="8"/>
-      <c r="AD1" s="7" t="s">
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="7"/>
+      <c r="AB1" s="7"/>
+      <c r="AD1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
+      <c r="AE1" s="7"/>
+      <c r="AF1" s="7"/>
+      <c r="AG1" s="7"/>
     </row>
     <row r="2" spans="1:33" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -1015,18 +1023,18 @@
       </c>
     </row>
     <row r="7" spans="1:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="G7" s="7" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="G7" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
       <c r="O7" s="9" t="s">
         <v>19</v>
       </c>
@@ -1130,8 +1138,12 @@
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="3"/>
+      <c r="B9" s="5">
+        <v>0.445851</v>
+      </c>
+      <c r="C9" s="3">
+        <v>1.4243299999999999E-3</v>
+      </c>
       <c r="D9" s="3">
         <v>9.5</v>
       </c>
@@ -1185,12 +1197,12 @@
       </c>
     </row>
     <row r="10" spans="1:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
       <c r="O10" s="9" t="s">
         <v>20</v>
       </c>
@@ -1217,16 +1229,12 @@
       <c r="AG10" s="10"/>
     </row>
     <row r="11" spans="1:33" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
       <c r="O11" s="4" t="s">
         <v>0</v>
       </c>
@@ -1277,12 +1285,12 @@
       </c>
     </row>
     <row r="12" spans="1:33" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
       <c r="G12" s="4" t="s">
         <v>0</v>
       </c>
@@ -1386,17 +1394,21 @@
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="3"/>
+      <c r="B14" s="5">
+        <v>8.8170899999999996E-2</v>
+      </c>
+      <c r="C14" s="3">
+        <v>6.7944999999999995E-4</v>
+      </c>
       <c r="D14" s="3">
         <v>9.5</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
       <c r="O14" s="4" t="s">
         <v>0</v>
       </c>
@@ -1447,12 +1459,12 @@
       </c>
     </row>
     <row r="15" spans="1:33" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
       <c r="O15" s="3" t="s">
         <v>3</v>
       </c>
@@ -1491,10 +1503,6 @@
       </c>
     </row>
     <row r="16" spans="1:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
       <c r="O16" s="9" t="s">
         <v>22</v>
       </c>
@@ -1521,12 +1529,12 @@
       <c r="AG16" s="10"/>
     </row>
     <row r="17" spans="1:33" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
       <c r="O17" s="4" t="s">
         <v>0</v>
       </c>
@@ -1630,8 +1638,12 @@
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="3"/>
+      <c r="B19" s="5">
+        <v>1.07243</v>
+      </c>
+      <c r="C19" s="3">
+        <v>3.9225600000000003E-3</v>
+      </c>
       <c r="D19" s="3">
         <v>9.5</v>
       </c>
@@ -1661,12 +1673,12 @@
       <c r="AG19" s="10"/>
     </row>
     <row r="20" spans="1:33" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
       <c r="O20" s="4" t="s">
         <v>0</v>
       </c>
@@ -1755,36 +1767,36 @@
       </c>
     </row>
     <row r="22" spans="1:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="O22" s="6" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="O22" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="P22" s="6"/>
-      <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
-      <c r="T22" s="6" t="s">
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="T22" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="U22" s="6"/>
-      <c r="V22" s="6"/>
-      <c r="W22" s="6"/>
-      <c r="Y22" s="6" t="s">
+      <c r="U22" s="8"/>
+      <c r="V22" s="8"/>
+      <c r="W22" s="8"/>
+      <c r="Y22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="Z22" s="6"/>
-      <c r="AA22" s="6"/>
-      <c r="AB22" s="6"/>
-      <c r="AD22" s="6" t="s">
+      <c r="Z22" s="8"/>
+      <c r="AA22" s="8"/>
+      <c r="AB22" s="8"/>
+      <c r="AD22" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="AE22" s="6"/>
-      <c r="AF22" s="6"/>
-      <c r="AG22" s="6"/>
+      <c r="AE22" s="8"/>
+      <c r="AF22" s="8"/>
+      <c r="AG22" s="8"/>
     </row>
     <row r="23" spans="1:33" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
@@ -1804,22 +1816,70 @@
       <c r="A24" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="3"/>
+      <c r="B24" s="5">
+        <v>1.19211</v>
+      </c>
+      <c r="C24" s="3">
+        <v>4.1660500000000001E-3</v>
+      </c>
       <c r="D24" s="3">
         <v>9.5</v>
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.2">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+    </row>
+    <row r="27" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="44">
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="O1:R1"/>
+    <mergeCell ref="O4:R4"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="O10:R10"/>
+    <mergeCell ref="O13:R13"/>
+    <mergeCell ref="T1:W1"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="T10:W10"/>
+    <mergeCell ref="T13:W13"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="Y4:AB4"/>
+    <mergeCell ref="Y7:AB7"/>
+    <mergeCell ref="Y10:AB10"/>
+    <mergeCell ref="Y13:AB13"/>
+    <mergeCell ref="AD1:AG1"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="AD7:AG7"/>
+    <mergeCell ref="AD10:AG10"/>
+    <mergeCell ref="AD13:AG13"/>
+    <mergeCell ref="AD19:AG19"/>
+    <mergeCell ref="AD22:AG22"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="AD16:AG16"/>
+    <mergeCell ref="T19:W19"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="Y16:AB16"/>
+    <mergeCell ref="Y19:AB19"/>
+    <mergeCell ref="Y22:AB22"/>
+    <mergeCell ref="T16:W16"/>
+    <mergeCell ref="O22:R22"/>
+    <mergeCell ref="O16:R16"/>
+    <mergeCell ref="O19:R19"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="A25:D25"/>
@@ -1828,49 +1888,34 @@
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A20:D20"/>
-    <mergeCell ref="AD19:AG19"/>
-    <mergeCell ref="AD22:AG22"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="AD1:AG1"/>
-    <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="AD7:AG7"/>
-    <mergeCell ref="AD10:AG10"/>
-    <mergeCell ref="AD13:AG13"/>
-    <mergeCell ref="AD16:AG16"/>
-    <mergeCell ref="T19:W19"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="Y4:AB4"/>
-    <mergeCell ref="Y7:AB7"/>
-    <mergeCell ref="Y10:AB10"/>
-    <mergeCell ref="Y13:AB13"/>
-    <mergeCell ref="Y16:AB16"/>
-    <mergeCell ref="Y19:AB19"/>
-    <mergeCell ref="Y22:AB22"/>
-    <mergeCell ref="T1:W1"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="T7:W7"/>
-    <mergeCell ref="T10:W10"/>
-    <mergeCell ref="T13:W13"/>
-    <mergeCell ref="T16:W16"/>
-    <mergeCell ref="O22:R22"/>
-    <mergeCell ref="O1:R1"/>
-    <mergeCell ref="O4:R4"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="O10:R10"/>
-    <mergeCell ref="O13:R13"/>
-    <mergeCell ref="O16:R16"/>
-    <mergeCell ref="O19:R19"/>
   </mergeCells>
+  <conditionalFormatting sqref="N7 B9 B14 B19 B24 H13 H9 P3 P6 P9 P12 P15 P18 P21">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95316306-EFB9-4052-9201-767301A3C05F}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8.83203125" style="2"/>
@@ -1929,6 +1974,25 @@
         <v>16</v>
       </c>
     </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.91100300000000001</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1.41151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="2">
+        <v>1.8100499999999999E-3</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2.6979600000000001E-3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>